<commit_message>
Use checkbox glyphs instead of boolean for issue category
</commit_message>
<xml_diff>
--- a/02. FAT_Resolution Document/S4_FAT_AXCELEFT-3250_Runtime error during TECO of the workorder.xlsx
+++ b/02. FAT_Resolution Document/S4_FAT_AXCELEFT-3250_Runtime error during TECO of the workorder.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +108,12 @@
       <color rgb="FF555555"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI Symbol"/>
+      <b val="1"/>
+      <color rgb="FF7B0C0C"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -267,7 +273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -505,6 +511,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1094,8 +1103,10 @@
     </row>
     <row r="20" ht="21.95" customHeight="1">
       <c r="A20" s="10" t="n"/>
-      <c r="B20" s="13" t="b">
-        <v>0</v>
+      <c r="B20" s="86" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
@@ -1112,8 +1123,10 @@
     </row>
     <row r="21" ht="35.1" customHeight="1">
       <c r="A21" s="11" t="n"/>
-      <c r="B21" s="13" t="b">
-        <v>0</v>
+      <c r="B21" s="86" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
@@ -1131,8 +1144,10 @@
     </row>
     <row r="22" ht="35.1" customHeight="1">
       <c r="A22" s="10" t="n"/>
-      <c r="B22" s="13" t="b">
-        <v>1</v>
+      <c r="B22" s="86" t="inlineStr">
+        <is>
+          <t>☑</t>
+        </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
@@ -1150,8 +1165,10 @@
     </row>
     <row r="23" ht="21.95" customHeight="1">
       <c r="A23" s="11" t="n"/>
-      <c r="B23" s="13" t="b">
-        <v>0</v>
+      <c r="B23" s="86" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
@@ -1168,8 +1185,10 @@
     </row>
     <row r="24" ht="35.1" customHeight="1">
       <c r="A24" s="10" t="n"/>
-      <c r="B24" s="13" t="b">
-        <v>0</v>
+      <c r="B24" s="86" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
@@ -1186,8 +1205,10 @@
     </row>
     <row r="25" ht="21.95" customHeight="1">
       <c r="A25" s="11" t="n"/>
-      <c r="B25" s="13" t="b">
-        <v>0</v>
+      <c r="B25" s="86" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
@@ -1204,8 +1225,10 @@
     </row>
     <row r="26" ht="27.95" customHeight="1">
       <c r="A26" s="11" t="n"/>
-      <c r="B26" s="13" t="b">
-        <v>0</v>
+      <c r="B26" s="86" t="inlineStr">
+        <is>
+          <t>☐</t>
+        </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
         <is>

</xml_diff>